<commit_message>
feat(ui): sidebar retrátil com ícones + script seed/set-test-phone
- Sidebar com toggle PanelLeftClose/Open, persiste em localStorage
- Ícones Lucide para cada item de navegação
- Telefones do template apontam para +4740346834 (telefone de teste do dev)
- Script scripts/set-test-phone.ts para atualizar clientes existentes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/surfsup-conversion-template.xlsx
+++ b/templates/surfsup-conversion-template.xlsx
@@ -484,7 +484,7 @@
         <v>João Pereira</v>
       </c>
       <c r="L2" t="str">
-        <v>+5511991234567</v>
+        <v>+4740346834</v>
       </c>
       <c r="M2" t="str">
         <v>joao@example.com</v>
@@ -531,7 +531,7 @@
         <v>Maria Souza</v>
       </c>
       <c r="L3" t="str">
-        <v>+5521987654321</v>
+        <v>+4740346834</v>
       </c>
       <c r="M3" t="str">
         <v>maria@example.com</v>
@@ -578,7 +578,7 @@
         <v>João Pereira</v>
       </c>
       <c r="L4" t="str">
-        <v>+5511991234567</v>
+        <v>+4740346834</v>
       </c>
       <c r="M4" t="str">
         <v>joao@example.com</v>
@@ -628,7 +628,7 @@
         <v>Ana Carolina Lima</v>
       </c>
       <c r="L5" t="str">
-        <v>11955554444</v>
+        <v>+4740346834</v>
       </c>
       <c r="N5" t="str">
         <v>12-03-2026</v>
@@ -672,7 +672,7 @@
         <v>Bruno Carvalho</v>
       </c>
       <c r="L6" t="str">
-        <v>+5511966667777</v>
+        <v>+4740346834</v>
       </c>
       <c r="M6" t="str">
         <v>bruno@example.com</v>

</xml_diff>